<commit_message>
ANW-3030 Describe the Archival Object import rep/nonrep columns as Display Thumbnail/Link
The rep_* columns create the Display Thumbnail file version and the nonrep_*
columns the Display Link one. Only the labels change: the column codes stay,
so existing spreadsheets keep working. The nonrep_publish label notes that only
a published file version becomes the Display Link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_template.xlsx
@@ -204,67 +204,67 @@
 (Note that Publish value will be inherited by each File Version in addition to being set on the Digital Object record. Leave this blank to get the default value FALSE.)</t>
   </si>
   <si>
-    <t>Linked-to URL for representative file version</t>
-  </si>
-  <si>
-    <t>Use Statement for representative file version</t>
-  </si>
-  <si>
-    <t>Xlink actuate attribute for representative file version (previous default 'onRequest')</t>
-  </si>
-  <si>
-    <t>Xlink show attribute for representative file version (previous default 'new')</t>
-  </si>
-  <si>
-    <t>File Format Name for representative file version</t>
-  </si>
-  <si>
-    <t>File Format Version for representative file version</t>
-  </si>
-  <si>
-    <t>File size (bytes) for representative file version</t>
-  </si>
-  <si>
-    <t>Checksum for representative file version</t>
-  </si>
-  <si>
-    <t>Checksum Method for representative file version</t>
-  </si>
-  <si>
-    <t>Caption for representative file version</t>
-  </si>
-  <si>
-    <t>Linked-to URL for non-representative file version</t>
-  </si>
-  <si>
-    <t>Publish non-representative file version?</t>
-  </si>
-  <si>
-    <t>Use Statement for non-representative file version</t>
-  </si>
-  <si>
-    <t>Xlink actuate attribute for non-representative file version (previous default 'onLoad')</t>
-  </si>
-  <si>
-    <t>Xlink show attribute for non-representative file version (previous default 'embed')</t>
-  </si>
-  <si>
-    <t>File Format Name for non-representative file version</t>
-  </si>
-  <si>
-    <t>File Format Version for non-representative file version</t>
-  </si>
-  <si>
-    <t>File size (bytes) for non-representative file version</t>
-  </si>
-  <si>
-    <t>Checksum for non-representative file version</t>
-  </si>
-  <si>
-    <t>Checksum Method for non-representative file version</t>
-  </si>
-  <si>
-    <t>Caption for non-representative file version</t>
+    <t>Linked-to URL for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Use Statement for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Xlink actuate attribute for Display Thumbnail file version (previous default 'onRequest')</t>
+  </si>
+  <si>
+    <t>Xlink show attribute for Display Thumbnail file version (previous default 'new')</t>
+  </si>
+  <si>
+    <t>File Format Name for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>File Format Version for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>File size (bytes) for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Checksum for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Checksum Method for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Caption for Display Thumbnail file version</t>
+  </si>
+  <si>
+    <t>Linked-to URL for Display Link file version</t>
+  </si>
+  <si>
+    <t>Publish the Display Link file version? (only a published file version becomes the Display Link)</t>
+  </si>
+  <si>
+    <t>Use Statement for Display Link file version</t>
+  </si>
+  <si>
+    <t>Xlink actuate attribute for Display Link file version (previous default 'onLoad')</t>
+  </si>
+  <si>
+    <t>Xlink show attribute for Display Link file version (previous default 'embed')</t>
+  </si>
+  <si>
+    <t>File Format Name for Display Link file version</t>
+  </si>
+  <si>
+    <t>File Format Version for Display Link file version</t>
+  </si>
+  <si>
+    <t>File size (bytes) for Display Link file version</t>
+  </si>
+  <si>
+    <t>Checksum for Display Link file version</t>
+  </si>
+  <si>
+    <t>Checksum Method for Display Link file version</t>
+  </si>
+  <si>
+    <t>Caption for Display Link file version</t>
   </si>
   <si>
     <t>Person Agent Record ID
@@ -1197,7 +1197,7 @@
     <t>Publish Digital Object Record</t>
   </si>
   <si>
-    <t>URL of representative file version</t>
+    <t>URL of Display Thumbnail file version</t>
   </si>
   <si>
     <t>Use Statement</t>
@@ -1227,7 +1227,7 @@
     <t>Caption</t>
   </si>
   <si>
-    <t>URL of non-representative file version</t>
+    <t>URL of Display Link file version</t>
   </si>
   <si>
     <t>Publish</t>

</xml_diff>